<commit_message>
included more allocation rooms
</commit_message>
<xml_diff>
--- a/uploads/class_strength.xlsx
+++ b/uploads/class_strength.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCD9E6C-1DC4-48BE-A452-B5B86ABF1DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B0E932-FF39-4067-AB68-934F75FF4E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04AEA855-3334-4620-AE19-CA8C89032C65}"/>
   </bookViews>
@@ -516,7 +516,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -527,7 +527,7 @@
         <v>29</v>
       </c>
       <c r="B3">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
@@ -538,7 +538,7 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -549,7 +549,7 @@
         <v>2</v>
       </c>
       <c r="B5">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
@@ -560,7 +560,7 @@
         <v>3</v>
       </c>
       <c r="B6">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
@@ -571,7 +571,7 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -582,7 +582,7 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -593,7 +593,7 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
         <v>28</v>
@@ -604,7 +604,7 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
@@ -615,7 +615,7 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
         <v>28</v>
@@ -648,7 +648,7 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
         <v>28</v>
@@ -659,7 +659,7 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
         <v>28</v>
@@ -681,7 +681,7 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
         <v>28</v>
@@ -692,7 +692,7 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
         <v>28</v>
@@ -714,7 +714,7 @@
         <v>21</v>
       </c>
       <c r="B20">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
         <v>28</v>
@@ -725,7 +725,7 @@
         <v>22</v>
       </c>
       <c r="B21">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
         <v>28</v>
@@ -736,7 +736,7 @@
         <v>23</v>
       </c>
       <c r="B22">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
         <v>28</v>
@@ -747,7 +747,7 @@
         <v>24</v>
       </c>
       <c r="B23">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
         <v>28</v>

</xml_diff>